<commit_message>
docs: sync final WBS and submission status
</commit_message>
<xml_diff>
--- a/outputs/Procurement_WBS_v1.3.xlsx
+++ b/outputs/Procurement_WBS_v1.3.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" r:id="Re9a5a0a1825c45dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracking" sheetId="2" r:id="R76ae6f36fb794979"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" r:id="Rc384e69659694d19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracking" sheetId="2" r:id="R690c87fb39664ce5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -581,14 +581,14 @@
       </x:c>
       <x:c r="D4" s="9" t="n">
         <x:f>COUNTIFS(B9:B42,2,H9:H42,"Terverifikasi")</x:f>
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E4" s="7" t="s">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F4" s="8" t="n">
         <x:f>COUNTIFS(B9:B42,2,H9:H42,"Dikerjakan")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="7" t="str">
         <x:v>Disetujui</x:v>
@@ -612,7 +612,7 @@
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
       <x:c r="A6" s="22" t="str">
-        <x:v>Setup bersih versi akhir lulus. Pemeriksaan akhir konfigurasi server dan commit/push penyerahan masih terbuka.</x:v>
+        <x:v>Setup, pemeriksaan hosting, dan commit/push sumber terverifikasi. Pengiriman lampiran serta informasi akses belum dikonfirmasi.</x:v>
       </x:c>
       <x:c r="B6" s="22"/>
       <x:c r="C6" s="22"/>
@@ -1389,7 +1389,7 @@
         <x:v>Verifikasi keamanan dasar</x:v>
       </x:c>
       <x:c r="D39" s="16" t="str">
-        <x:v>Pemeriksaan lokal dan publik hosting lulus: HTTPS/header, CSRF, route privat dan delapan aset. Pemeriksaan akhir konfigurasi/izin file pada server masih terbuka.</x:v>
+        <x:v>Pemeriksaan keamanan dasar lokal dan hosting lulus pada lingkup tercatat: HTTPS/header, CSRF, akses, migrasi dan izin file privat. Dua warning HSTS terdokumentasi.</x:v>
       </x:c>
       <x:c r="E39" s="16" t="str">
         <x:v>Engineer</x:v>
@@ -1401,7 +1401,7 @@
         <x:v>6.1; 6.2</x:v>
       </x:c>
       <x:c r="H39" s="16" t="str">
-        <x:v>Dikerjakan</x:v>
+        <x:v>Terverifikasi</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="92" customHeight="1">
@@ -1415,7 +1415,7 @@
         <x:v>Paket penyerahan</x:v>
       </x:c>
       <x:c r="D40" s="4" t="str">
-        <x:v>Paket sumber terbaru, manifest, panduan penyerahan dan lampiran siap. GitHub publik masih commit e07f790; commit/push serta verifikasi hasil penyerahan dilakukan pengguna.</x:v>
+        <x:v>Sumber pada main commit 5209c62 sudah dipush dan diverifikasi. Lampiran tersedia pada repository; pengiriman hasil melalui email belum dikonfirmasi.</x:v>
       </x:c>
       <x:c r="E40" s="4" t="str">
         <x:v>Engineer</x:v>
@@ -1494,7 +1494,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d3966b9357c4039"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffcae01c12f24b3a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1612,7 +1612,7 @@
         <x:v>Seluruh BP/GW</x:v>
       </x:c>
       <x:c r="D8" s="16" t="str">
-        <x:v>27 paket; dependensi acyclic; formula ringkasan dan status Tracking diuji dengan perubahan lalu dipulihkan.</x:v>
+        <x:v>27 paket; dependensi tidak bersiklus; formula ringkasan dan status Tracking diuji dengan perubahan lalu dipulihkan.</x:v>
       </x:c>
       <x:c r="E8" s="16" t="str">
         <x:v>Dokumen perencanaan</x:v>
@@ -2095,14 +2095,14 @@
         <x:v>BP-00; BP-02; BP-13</x:v>
       </x:c>
       <x:c r="D31" s="4" t="str">
-        <x:v>HTTPS/header/CSRF; lima route login, lima lokasi privat 404, delapan hash static cocok. Console host belum menuntaskan check --deploy dan izin file privat.</x:v>
+        <x:v>Screenshot hosting: check --deploy hanya W005/W021, migrate --check tanpa error, izin folder privat 700 dan kedua file 600. Pemeriksaan HTTP/aset lulus.</x:v>
       </x:c>
       <x:c r="E31" s="4" t="str">
         <x:v>Kebutuhan produk</x:v>
       </x:c>
       <x:c r="F31" s="4" t="str">
         <x:f>WBS!H39</x:f>
-        <x:v>Dikerjakan</x:v>
+        <x:v>Terverifikasi</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="92" customHeight="1">
@@ -2116,7 +2116,7 @@
         <x:v>Seluruh proses</x:v>
       </x:c>
       <x:c r="D32" s="16" t="str">
-        <x:v>Paket lokal diperiksa; remote publik masih tanpa dependensi AI. Finalisasi menunggu pemeriksaan server, commit/push pengguna dan pencocokan hasil di GitHub.</x:v>
+        <x:v>Remote main 5209c62 sudah diverifikasi. Paket dan lampiran tersedia; pengiriman lampiran serta informasi akses melalui email belum dikonfirmasi.</x:v>
       </x:c>
       <x:c r="E32" s="16" t="str">
         <x:v>Kelengkapan penyerahan</x:v>
@@ -2161,7 +2161,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5531941b0c6b459e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe368f3dce9e4704"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>